<commit_message>
Add Gantt chart visualization
Stacked bar chart on a new sheet, driven by タスク一覧's computed
start/end dates and critical-path flag (critical tasks shown in red).
</commit_message>
<xml_diff>
--- a/progress_tracker.xlsx
+++ b/progress_tracker.xlsx
@@ -14,6 +14,7 @@
     <sheet name="担当者一覧" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="タスク一覧" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="ダッシュボード" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="ガントチャート" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">タスク一覧!$A$2:$S$102</definedName>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="120">
   <si>
     <t xml:space="preserve">進捗管理シート 使い方</t>
   </si>
@@ -165,6 +166,77 @@
   </si>
   <si>
     <t xml:space="preserve">担当者別・マイルストーン別の残タスク状況、プロジェクト全体の状況を自動集計します。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ガントチャート</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">「タスク一覧」の先頭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">件を線表</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">バーチャート</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">で可視化します。クリティカルパス上のタスクは赤、それ以外は青で表示されます。「タスク一覧」を更新すると自動的に反映されます。</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">■ タスク一覧の入力方法</t>
@@ -2656,6 +2728,306 @@
   </si>
   <si>
     <t xml:space="preserve">プロジェクト終了予定日</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">「タスク一覧」の先頭</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">件を表示します</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">グラフの元データは</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">D</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">F</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">列</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">計画開始日</t>
+  </si>
+  <si>
+    <t xml:space="preserve">計画終了日</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">オフセット日数
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">グラフ用</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">通常期間</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">グラフ用</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">クリティカル期間</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">グラフ用</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2669,7 +3041,7 @@
     <numFmt numFmtId="167" formatCode="General"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2782,6 +3154,40 @@
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -2799,7 +3205,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF305496"/>
-        <bgColor rgb="FF0066CC"/>
+        <bgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
     <fill>
@@ -3047,7 +3453,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFC00000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -3060,7 +3466,7 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
-      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFF2F2F2"/>
@@ -3068,7 +3474,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -3085,7 +3491,7 @@
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFC7CE"/>
-      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF4472C4"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
@@ -3106,8 +3512,818 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>ガントチャート(計画開始日〜計画終了日)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>" "</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v> </c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>ガントチャート!$A$5:$A$24</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>要件ヒアリング</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>要件定義書作成</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>要件レビュー</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>画面設計</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>DB設計</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>API設計</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>設計レビュー</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>実装</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>実装(画面)</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>テスト</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>リリース判定</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v/>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>ガントチャート!$D$5:$D$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"通常タスク"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>通常タスク</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4472c4"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>ガントチャート!$A$5:$A$24</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>要件ヒアリング</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>要件定義書作成</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>要件レビュー</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>画面設計</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>DB設計</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>API設計</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>設計レビュー</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>実装</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>実装(画面)</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>テスト</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>リリース判定</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v/>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>ガントチャート!$E$5:$E$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"クリティカルパス"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>クリティカルパス</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="c00000"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>ガントチャート!$A$5:$A$24</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>要件ヒアリング</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>要件定義書作成</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>要件レビュー</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>画面設計</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>DB設計</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>API設計</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>設計レビュー</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>実装</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>実装(画面)</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>テスト</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>リリース判定</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v/>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>ガントチャート!$F$5:$F$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="71290635"/>
+        <c:axId val="18685504"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="71290635"/>
+        <c:scaling>
+          <c:orientation val="maxMin"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="18685504"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="18685504"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>経過日数(プロジェクト開始日からの日数)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="71290635"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>58320</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>421920</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>61200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="0" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="4572000"/>
+        <a:ext cx="9359640" cy="6479640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3290,7 +4506,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:B56"/>
+  <dimension ref="B1:B58"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -3379,29 +4595,29 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="2"/>
+      <c r="B19" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="6" t="s">
-        <v>16</v>
-      </c>
+      <c r="B21" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="4" t="s">
         <v>19</v>
       </c>
@@ -3411,7 +4627,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
         <v>21</v>
       </c>
@@ -3421,7 +4637,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="4" t="s">
         <v>23</v>
       </c>
@@ -3437,20 +4653,20 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="2"/>
+      <c r="B32" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="4" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="3" t="s">
-        <v>27</v>
-      </c>
+      <c r="B34" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="5" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3505,39 +4721,49 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="2"/>
+      <c r="B47" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B48" s="4" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="4" t="s">
+      <c r="B49" s="2"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="5" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="2"/>
+    <row r="54" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B55" s="4" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="5" t="s">
-        <v>44</v>
+      <c r="B56" s="2"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -3566,35 +4792,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46237</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">IFERROR(MAX(タスク一覧!$L$3:$L$102),"")</f>
         <v>46280</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="true">TODAY()</f>
@@ -3633,58 +4859,58 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C3" s="14" t="n">
         <v>46248</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C4" s="14" t="n">
         <v>46276</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C5" s="14" t="n">
         <v>46304</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3731,7 +4957,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -3765,46 +4991,46 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B4" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>67</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3844,7 +5070,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -3888,61 +5114,61 @@
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K2" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="L2" s="11" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="M2" s="11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O2" s="11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="P2" s="11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="Q2" s="11" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="R2" s="11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="S2" s="11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3951,13 +5177,13 @@
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="13" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
@@ -3966,7 +5192,7 @@
         <v>3</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K3" s="19" t="n">
         <f aca="false">IF($A3="","",設定!$B$2)</f>
@@ -4011,13 +5237,13 @@
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F4" s="12" t="n">
         <v>1</v>
@@ -4028,7 +5254,7 @@
         <v>4</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K4" s="19" t="n">
         <f aca="false">IF($A4="","",IF(AND($F4="",$G4="",$H4=""),設定!$B$2,MAX(IF($F4="",0,IFERROR(WORKDAY(INDEX($L$3:$L$3,MATCH($F4,$A$3:$A$3,0)),1),0)),IF($G4="",0,IFERROR(WORKDAY(INDEX($L$3:$L$3,MATCH($G4,$A$3:$A$3,0)),1),0)),IF($H4="",0,IFERROR(WORKDAY(INDEX($L$3:$L$3,MATCH($H4,$A$3:$A$3,0)),1),0)))))</f>
@@ -4073,13 +5299,13 @@
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F5" s="12" t="n">
         <v>2</v>
@@ -4090,7 +5316,7 @@
         <v>2</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K5" s="19" t="n">
         <f aca="false">IF($A5="","",IF(AND($F5="",$G5="",$H5=""),設定!$B$2,MAX(IF($F5="",0,IFERROR(WORKDAY(INDEX($L$3:$L$4,MATCH($F5,$A$3:$A$4,0)),1),0)),IF($G5="",0,IFERROR(WORKDAY(INDEX($L$3:$L$4,MATCH($G5,$A$3:$A$4,0)),1),0)),IF($H5="",0,IFERROR(WORKDAY(INDEX($L$3:$L$4,MATCH($H5,$A$3:$A$4,0)),1),0)))))</f>
@@ -4135,13 +5361,13 @@
       </c>
       <c r="B6" s="12"/>
       <c r="C6" s="13" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F6" s="12" t="n">
         <v>3</v>
@@ -4152,7 +5378,7 @@
         <v>5</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K6" s="19" t="n">
         <f aca="false">IF($A6="","",IF(AND($F6="",$G6="",$H6=""),設定!$B$2,MAX(IF($F6="",0,IFERROR(WORKDAY(INDEX($L$3:$L$5,MATCH($F6,$A$3:$A$5,0)),1),0)),IF($G6="",0,IFERROR(WORKDAY(INDEX($L$3:$L$5,MATCH($G6,$A$3:$A$5,0)),1),0)),IF($H6="",0,IFERROR(WORKDAY(INDEX($L$3:$L$5,MATCH($H6,$A$3:$A$5,0)),1),0)))))</f>
@@ -4197,13 +5423,13 @@
       </c>
       <c r="B7" s="12"/>
       <c r="C7" s="12" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F7" s="12" t="n">
         <v>3</v>
@@ -4214,7 +5440,7 @@
         <v>5</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K7" s="19" t="n">
         <f aca="false">IF($A7="","",IF(AND($F7="",$G7="",$H7=""),設定!$B$2,MAX(IF($F7="",0,IFERROR(WORKDAY(INDEX($L$3:$L$6,MATCH($F7,$A$3:$A$6,0)),1),0)),IF($G7="",0,IFERROR(WORKDAY(INDEX($L$3:$L$6,MATCH($G7,$A$3:$A$6,0)),1),0)),IF($H7="",0,IFERROR(WORKDAY(INDEX($L$3:$L$6,MATCH($H7,$A$3:$A$6,0)),1),0)))))</f>
@@ -4259,13 +5485,13 @@
       </c>
       <c r="B8" s="12"/>
       <c r="C8" s="12" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F8" s="12" t="n">
         <v>5</v>
@@ -4276,7 +5502,7 @@
         <v>3</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K8" s="19" t="n">
         <f aca="false">IF($A8="","",IF(AND($F8="",$G8="",$H8=""),設定!$B$2,MAX(IF($F8="",0,IFERROR(WORKDAY(INDEX($L$3:$L$7,MATCH($F8,$A$3:$A$7,0)),1),0)),IF($G8="",0,IFERROR(WORKDAY(INDEX($L$3:$L$7,MATCH($G8,$A$3:$A$7,0)),1),0)),IF($H8="",0,IFERROR(WORKDAY(INDEX($L$3:$L$7,MATCH($H8,$A$3:$A$7,0)),1),0)))))</f>
@@ -4321,13 +5547,13 @@
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F9" s="12" t="n">
         <v>4</v>
@@ -4340,7 +5566,7 @@
         <v>2</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K9" s="19" t="n">
         <f aca="false">IF($A9="","",IF(AND($F9="",$G9="",$H9=""),設定!$B$2,MAX(IF($F9="",0,IFERROR(WORKDAY(INDEX($L$3:$L$8,MATCH($F9,$A$3:$A$8,0)),1),0)),IF($G9="",0,IFERROR(WORKDAY(INDEX($L$3:$L$8,MATCH($G9,$A$3:$A$8,0)),1),0)),IF($H9="",0,IFERROR(WORKDAY(INDEX($L$3:$L$8,MATCH($H9,$A$3:$A$8,0)),1),0)))))</f>
@@ -4385,13 +5611,13 @@
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F10" s="12" t="n">
         <v>7</v>
@@ -4402,7 +5628,7 @@
         <v>8</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K10" s="19" t="n">
         <f aca="false">IF($A10="","",IF(AND($F10="",$G10="",$H10=""),設定!$B$2,MAX(IF($F10="",0,IFERROR(WORKDAY(INDEX($L$3:$L$9,MATCH($F10,$A$3:$A$9,0)),1),0)),IF($G10="",0,IFERROR(WORKDAY(INDEX($L$3:$L$9,MATCH($G10,$A$3:$A$9,0)),1),0)),IF($H10="",0,IFERROR(WORKDAY(INDEX($L$3:$L$9,MATCH($H10,$A$3:$A$9,0)),1),0)))))</f>
@@ -4449,13 +5675,13 @@
         <v>8</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
@@ -4464,7 +5690,7 @@
         <v>4</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K11" s="19" t="n">
         <f aca="false">IF($A11="","",IF(AND($F11="",$G11="",$H11=""),設定!$B$2,MAX(IF($F11="",0,IFERROR(WORKDAY(INDEX($L$3:$L$10,MATCH($F11,$A$3:$A$10,0)),1),0)),IF($G11="",0,IFERROR(WORKDAY(INDEX($L$3:$L$10,MATCH($G11,$A$3:$A$10,0)),1),0)),IF($H11="",0,IFERROR(WORKDAY(INDEX($L$3:$L$10,MATCH($H11,$A$3:$A$10,0)),1),0)))))</f>
@@ -4509,13 +5735,13 @@
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F12" s="12" t="n">
         <v>8</v>
@@ -4526,7 +5752,7 @@
         <v>4</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K12" s="19" t="n">
         <f aca="false">IF($A12="","",IF(AND($F12="",$G12="",$H12=""),設定!$B$2,MAX(IF($F12="",0,IFERROR(WORKDAY(INDEX($L$3:$L$11,MATCH($F12,$A$3:$A$11,0)),1),0)),IF($G12="",0,IFERROR(WORKDAY(INDEX($L$3:$L$11,MATCH($G12,$A$3:$A$11,0)),1),0)),IF($H12="",0,IFERROR(WORKDAY(INDEX($L$3:$L$11,MATCH($H12,$A$3:$A$11,0)),1),0)))))</f>
@@ -4571,13 +5797,13 @@
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="13" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F13" s="12" t="n">
         <v>9</v>
@@ -4588,7 +5814,7 @@
         <v>1</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K13" s="19" t="n">
         <f aca="false">IF($A13="","",IF(AND($F13="",$G13="",$H13=""),設定!$B$2,MAX(IF($F13="",0,IFERROR(WORKDAY(INDEX($L$3:$L$12,MATCH($F13,$A$3:$A$12,0)),1),0)),IF($G13="",0,IFERROR(WORKDAY(INDEX($L$3:$L$12,MATCH($G13,$A$3:$A$12,0)),1),0)),IF($H13="",0,IFERROR(WORKDAY(INDEX($L$3:$L$12,MATCH($H13,$A$3:$A$12,0)),1),0)))))</f>
@@ -8960,21 +10186,21 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9159,27 +10385,27 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9444,12 +10670,12 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="25" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B30" s="23" t="n">
         <f aca="false">COUNT(タスク一覧!$A$3:$A$102)</f>
@@ -9458,7 +10684,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="25" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B31" s="23" t="n">
         <f aca="false">SUM(タスク一覧!$S$3:$S$102)</f>
@@ -9467,7 +10693,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="25" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B32" s="23" t="n">
         <f aca="false">COUNTIFS(タスク一覧!$P$3:$P$102,"クリティカル",タスク一覧!$S$3:$S$102,1)</f>
@@ -9476,7 +10702,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="25" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B33" s="23" t="n">
         <f aca="false">COUNTIF(タスク一覧!$Q$3:$Q$102,"遅延")</f>
@@ -9485,7 +10711,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="25" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B34" s="9" t="n">
         <f aca="false">設定!$B$2</f>
@@ -9494,7 +10720,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="25" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B35" s="9" t="n">
         <f aca="false">設定!$B$3</f>
@@ -9510,4 +10736,580 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="38.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$3="","",タスク一覧!$C$3)</f>
+        <v>要件ヒアリング</v>
+      </c>
+      <c r="B5" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$3="","",タスク一覧!$K$3)</f>
+        <v>46237</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$3="","",タスク一覧!$L$3)</f>
+        <v>46239</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$3="",0,タスク一覧!$K$3-設定!$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$3="",0,IF(タスク一覧!$P$3="クリティカル",0,タスク一覧!$L$3-タスク一覧!$K$3+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$3="",0,IF(タスク一覧!$P$3="クリティカル",タスク一覧!$L$3-タスク一覧!$K$3+1,0))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$4="","",タスク一覧!$C$4)</f>
+        <v>要件定義書作成</v>
+      </c>
+      <c r="B6" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$4="","",タスク一覧!$K$4)</f>
+        <v>46240</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$4="","",タスク一覧!$L$4)</f>
+        <v>46245</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$4="",0,タスク一覧!$K$4-設定!$B$2)</f>
+        <v>3</v>
+      </c>
+      <c r="E6" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$4="",0,IF(タスク一覧!$P$4="クリティカル",0,タスク一覧!$L$4-タスク一覧!$K$4+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$4="",0,IF(タスク一覧!$P$4="クリティカル",タスク一覧!$L$4-タスク一覧!$K$4+1,0))</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$5="","",タスク一覧!$C$5)</f>
+        <v>要件レビュー</v>
+      </c>
+      <c r="B7" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$5="","",タスク一覧!$K$5)</f>
+        <v>46246</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$5="","",タスク一覧!$L$5)</f>
+        <v>46247</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$5="",0,タスク一覧!$K$5-設定!$B$2)</f>
+        <v>9</v>
+      </c>
+      <c r="E7" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$5="",0,IF(タスク一覧!$P$5="クリティカル",0,タスク一覧!$L$5-タスク一覧!$K$5+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$5="",0,IF(タスク一覧!$P$5="クリティカル",タスク一覧!$L$5-タスク一覧!$K$5+1,0))</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$6="","",タスク一覧!$C$6)</f>
+        <v>画面設計</v>
+      </c>
+      <c r="B8" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$6="","",タスク一覧!$K$6)</f>
+        <v>46248</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$6="","",タスク一覧!$L$6)</f>
+        <v>46254</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$6="",0,タスク一覧!$K$6-設定!$B$2)</f>
+        <v>11</v>
+      </c>
+      <c r="E8" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$6="",0,IF(タスク一覧!$P$6="クリティカル",0,タスク一覧!$L$6-タスク一覧!$K$6+1))</f>
+        <v>7</v>
+      </c>
+      <c r="F8" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$6="",0,IF(タスク一覧!$P$6="クリティカル",タスク一覧!$L$6-タスク一覧!$K$6+1,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$7="","",タスク一覧!$C$7)</f>
+        <v>DB設計</v>
+      </c>
+      <c r="B9" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$7="","",タスク一覧!$K$7)</f>
+        <v>46248</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$7="","",タスク一覧!$L$7)</f>
+        <v>46254</v>
+      </c>
+      <c r="D9" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$7="",0,タスク一覧!$K$7-設定!$B$2)</f>
+        <v>11</v>
+      </c>
+      <c r="E9" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$7="",0,IF(タスク一覧!$P$7="クリティカル",0,タスク一覧!$L$7-タスク一覧!$K$7+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$7="",0,IF(タスク一覧!$P$7="クリティカル",タスク一覧!$L$7-タスク一覧!$K$7+1,0))</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$8="","",タスク一覧!$C$8)</f>
+        <v>API設計</v>
+      </c>
+      <c r="B10" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$8="","",タスク一覧!$K$8)</f>
+        <v>46255</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$8="","",タスク一覧!$L$8)</f>
+        <v>46259</v>
+      </c>
+      <c r="D10" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$8="",0,タスク一覧!$K$8-設定!$B$2)</f>
+        <v>18</v>
+      </c>
+      <c r="E10" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$8="",0,IF(タスク一覧!$P$8="クリティカル",0,タスク一覧!$L$8-タスク一覧!$K$8+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$8="",0,IF(タスク一覧!$P$8="クリティカル",タスク一覧!$L$8-タスク一覧!$K$8+1,0))</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$9="","",タスク一覧!$C$9)</f>
+        <v>設計レビュー</v>
+      </c>
+      <c r="B11" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$9="","",タスク一覧!$K$9)</f>
+        <v>46260</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$9="","",タスク一覧!$L$9)</f>
+        <v>46261</v>
+      </c>
+      <c r="D11" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$9="",0,タスク一覧!$K$9-設定!$B$2)</f>
+        <v>23</v>
+      </c>
+      <c r="E11" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$9="",0,IF(タスク一覧!$P$9="クリティカル",0,タスク一覧!$L$9-タスク一覧!$K$9+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$9="",0,IF(タスク一覧!$P$9="クリティカル",タスク一覧!$L$9-タスク一覧!$K$9+1,0))</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$10="","",タスク一覧!$C$10)</f>
+        <v>実装</v>
+      </c>
+      <c r="B12" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$10="","",タスク一覧!$K$10)</f>
+        <v>46262</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$10="","",タスク一覧!$L$10)</f>
+        <v>46273</v>
+      </c>
+      <c r="D12" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$10="",0,タスク一覧!$K$10-設定!$B$2)</f>
+        <v>25</v>
+      </c>
+      <c r="E12" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$10="",0,IF(タスク一覧!$P$10="クリティカル",0,タスク一覧!$L$10-タスク一覧!$K$10+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$10="",0,IF(タスク一覧!$P$10="クリティカル",タスク一覧!$L$10-タスク一覧!$K$10+1,0))</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$11="","",タスク一覧!$C$11)</f>
+        <v>実装(画面)</v>
+      </c>
+      <c r="B13" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$11="","",タスク一覧!$K$11)</f>
+        <v>46237</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$11="","",タスク一覧!$L$11)</f>
+        <v>46240</v>
+      </c>
+      <c r="D13" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$11="",0,タスク一覧!$K$11-設定!$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$11="",0,IF(タスク一覧!$P$11="クリティカル",0,タスク一覧!$L$11-タスク一覧!$K$11+1))</f>
+        <v>4</v>
+      </c>
+      <c r="F13" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$11="",0,IF(タスク一覧!$P$11="クリティカル",タスク一覧!$L$11-タスク一覧!$K$11+1,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$12="","",タスク一覧!$C$12)</f>
+        <v>テスト</v>
+      </c>
+      <c r="B14" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$12="","",タスク一覧!$K$12)</f>
+        <v>46274</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$12="","",タスク一覧!$L$12)</f>
+        <v>46279</v>
+      </c>
+      <c r="D14" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$12="",0,タスク一覧!$K$12-設定!$B$2)</f>
+        <v>37</v>
+      </c>
+      <c r="E14" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$12="",0,IF(タスク一覧!$P$12="クリティカル",0,タスク一覧!$L$12-タスク一覧!$K$12+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$12="",0,IF(タスク一覧!$P$12="クリティカル",タスク一覧!$L$12-タスク一覧!$K$12+1,0))</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$13="","",タスク一覧!$C$13)</f>
+        <v>リリース判定</v>
+      </c>
+      <c r="B15" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$13="","",タスク一覧!$K$13)</f>
+        <v>46280</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$13="","",タスク一覧!$L$13)</f>
+        <v>46280</v>
+      </c>
+      <c r="D15" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$13="",0,タスク一覧!$K$13-設定!$B$2)</f>
+        <v>43</v>
+      </c>
+      <c r="E15" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$13="",0,IF(タスク一覧!$P$13="クリティカル",0,タスク一覧!$L$13-タスク一覧!$K$13+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$13="",0,IF(タスク一覧!$P$13="クリティカル",タスク一覧!$L$13-タスク一覧!$K$13+1,0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$14="","",タスク一覧!$C$14)</f>
+        <v/>
+      </c>
+      <c r="B16" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$14="","",タスク一覧!$K$14)</f>
+        <v/>
+      </c>
+      <c r="C16" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$14="","",タスク一覧!$L$14)</f>
+        <v/>
+      </c>
+      <c r="D16" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$14="",0,タスク一覧!$K$14-設定!$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$14="",0,IF(タスク一覧!$P$14="クリティカル",0,タスク一覧!$L$14-タスク一覧!$K$14+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$14="",0,IF(タスク一覧!$P$14="クリティカル",タスク一覧!$L$14-タスク一覧!$K$14+1,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$15="","",タスク一覧!$C$15)</f>
+        <v/>
+      </c>
+      <c r="B17" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$15="","",タスク一覧!$K$15)</f>
+        <v/>
+      </c>
+      <c r="C17" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$15="","",タスク一覧!$L$15)</f>
+        <v/>
+      </c>
+      <c r="D17" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$15="",0,タスク一覧!$K$15-設定!$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$15="",0,IF(タスク一覧!$P$15="クリティカル",0,タスク一覧!$L$15-タスク一覧!$K$15+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$15="",0,IF(タスク一覧!$P$15="クリティカル",タスク一覧!$L$15-タスク一覧!$K$15+1,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$16="","",タスク一覧!$C$16)</f>
+        <v/>
+      </c>
+      <c r="B18" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$16="","",タスク一覧!$K$16)</f>
+        <v/>
+      </c>
+      <c r="C18" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$16="","",タスク一覧!$L$16)</f>
+        <v/>
+      </c>
+      <c r="D18" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$16="",0,タスク一覧!$K$16-設定!$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$16="",0,IF(タスク一覧!$P$16="クリティカル",0,タスク一覧!$L$16-タスク一覧!$K$16+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$16="",0,IF(タスク一覧!$P$16="クリティカル",タスク一覧!$L$16-タスク一覧!$K$16+1,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$17="","",タスク一覧!$C$17)</f>
+        <v/>
+      </c>
+      <c r="B19" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$17="","",タスク一覧!$K$17)</f>
+        <v/>
+      </c>
+      <c r="C19" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$17="","",タスク一覧!$L$17)</f>
+        <v/>
+      </c>
+      <c r="D19" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$17="",0,タスク一覧!$K$17-設定!$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$17="",0,IF(タスク一覧!$P$17="クリティカル",0,タスク一覧!$L$17-タスク一覧!$K$17+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$17="",0,IF(タスク一覧!$P$17="クリティカル",タスク一覧!$L$17-タスク一覧!$K$17+1,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$18="","",タスク一覧!$C$18)</f>
+        <v/>
+      </c>
+      <c r="B20" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$18="","",タスク一覧!$K$18)</f>
+        <v/>
+      </c>
+      <c r="C20" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$18="","",タスク一覧!$L$18)</f>
+        <v/>
+      </c>
+      <c r="D20" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$18="",0,タスク一覧!$K$18-設定!$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$18="",0,IF(タスク一覧!$P$18="クリティカル",0,タスク一覧!$L$18-タスク一覧!$K$18+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$18="",0,IF(タスク一覧!$P$18="クリティカル",タスク一覧!$L$18-タスク一覧!$K$18+1,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$19="","",タスク一覧!$C$19)</f>
+        <v/>
+      </c>
+      <c r="B21" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$19="","",タスク一覧!$K$19)</f>
+        <v/>
+      </c>
+      <c r="C21" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$19="","",タスク一覧!$L$19)</f>
+        <v/>
+      </c>
+      <c r="D21" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$19="",0,タスク一覧!$K$19-設定!$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$19="",0,IF(タスク一覧!$P$19="クリティカル",0,タスク一覧!$L$19-タスク一覧!$K$19+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$19="",0,IF(タスク一覧!$P$19="クリティカル",タスク一覧!$L$19-タスク一覧!$K$19+1,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$20="","",タスク一覧!$C$20)</f>
+        <v/>
+      </c>
+      <c r="B22" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$20="","",タスク一覧!$K$20)</f>
+        <v/>
+      </c>
+      <c r="C22" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$20="","",タスク一覧!$L$20)</f>
+        <v/>
+      </c>
+      <c r="D22" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$20="",0,タスク一覧!$K$20-設定!$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E22" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$20="",0,IF(タスク一覧!$P$20="クリティカル",0,タスク一覧!$L$20-タスク一覧!$K$20+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$20="",0,IF(タスク一覧!$P$20="クリティカル",タスク一覧!$L$20-タスク一覧!$K$20+1,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$21="","",タスク一覧!$C$21)</f>
+        <v/>
+      </c>
+      <c r="B23" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$21="","",タスク一覧!$K$21)</f>
+        <v/>
+      </c>
+      <c r="C23" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$21="","",タスク一覧!$L$21)</f>
+        <v/>
+      </c>
+      <c r="D23" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$21="",0,タスク一覧!$K$21-設定!$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$21="",0,IF(タスク一覧!$P$21="クリティカル",0,タスク一覧!$L$21-タスク一覧!$K$21+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$21="",0,IF(タスク一覧!$P$21="クリティカル",タスク一覧!$L$21-タスク一覧!$K$21+1,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="23" t="str">
+        <f aca="false">IF(タスク一覧!$A$22="","",タスク一覧!$C$22)</f>
+        <v/>
+      </c>
+      <c r="B24" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$22="","",タスク一覧!$K$22)</f>
+        <v/>
+      </c>
+      <c r="C24" s="9" t="str">
+        <f aca="false">IF(タスク一覧!$A$22="","",タスク一覧!$L$22)</f>
+        <v/>
+      </c>
+      <c r="D24" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$22="",0,タスク一覧!$K$22-設定!$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$22="",0,IF(タスク一覧!$P$22="クリティカル",0,タスク一覧!$L$22-タスク一覧!$K$22+1))</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="23" t="n">
+        <f aca="false">IF(タスク一覧!$A$22="",0,IF(タスク一覧!$P$22="クリティカル",タスク一覧!$L$22-タスク一覧!$K$22+1,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Show real calendar dates on the Gantt chart's axis
Switch the chart's vertical axis from a day-offset count to actual
dates (weekly gridlines), with axis bounds sized to the sample
project's date range.
</commit_message>
<xml_diff>
--- a/progress_tracker.xlsx
+++ b/progress_tracker.xlsx
@@ -235,7 +235,64 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">で可視化します。クリティカルパス上のタスクは赤、それ以外は青で表示されます。「タスク一覧」を更新すると自動的に反映されます。</t>
+      <t xml:space="preserve">で可視化します。横軸は実際の日付です。クリティカルパス上のタスクは赤、それ以外は青で表示されます。「タスク一覧」を更新すると自動的に反映されます。★横軸</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">縦軸の目盛</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の表示範囲はサンプルのプロジェクト期間に合わせて固定されています。「設定」シートのプロジェクト開始日を大きく変更した場合は、グラフの縦軸を右クリック→「軸の書式設定」で最小値</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">最大値を実際の期間に合わせて調整してください。</t>
     </r>
   </si>
   <si>
@@ -2861,7 +2918,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">オフセット日数
+      <t xml:space="preserve">開始日シリアル値
 </t>
     </r>
     <r>
@@ -2884,6 +2941,27 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">グラフ用</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">非表示</t>
     </r>
     <r>
       <rPr>
@@ -3034,14 +3112,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="General"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="mm/dd"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3169,20 +3248,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="WenQuanYi Zen Hei"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -3675,40 +3740,40 @@
             <c:numRef>
               <c:f>ガントチャート!$D$5:$D$24</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>yyyy\-mm\-dd</c:formatCode>
                 <c:ptCount val="20"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>46237</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3</c:v>
+                  <c:v>46240</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9</c:v>
+                  <c:v>46246</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>11</c:v>
+                  <c:v>46248</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>11</c:v>
+                  <c:v>46248</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>18</c:v>
+                  <c:v>46255</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>23</c:v>
+                  <c:v>46260</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>25</c:v>
+                  <c:v>46262</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>46237</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>37</c:v>
+                  <c:v>46274</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>43</c:v>
+                  <c:v>46280</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -4115,11 +4180,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="71290635"/>
-        <c:axId val="18685504"/>
+        <c:axId val="55608121"/>
+        <c:axId val="51485318"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="71290635"/>
+        <c:axId val="55608121"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4151,7 +4216,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18685504"/>
+        <c:crossAx val="51485318"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4159,9 +4224,11 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="18685504"/>
+        <c:axId val="51485318"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="46283"/>
+          <c:min val="46234"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -4175,42 +4242,8 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t>経過日数(プロジェクト開始日からの日数)</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln w="0">
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:numFmt formatCode="mm/dd" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -4235,9 +4268,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71290635"/>
+        <c:crossAx val="55608121"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="7"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -4298,13 +4332,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>58320</xdr:rowOff>
+      <xdr:rowOff>39240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>421920</xdr:colOff>
       <xdr:row>56</xdr:row>
-      <xdr:rowOff>61200</xdr:rowOff>
+      <xdr:rowOff>42120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -4599,7 +4633,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="4" t="s">
         <v>16</v>
       </c>
@@ -10762,7 +10796,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="38.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
         <v>74</v>
       </c>
@@ -10795,9 +10829,9 @@
         <f aca="false">IF(タスク一覧!$A$3="","",タスク一覧!$L$3)</f>
         <v>46239</v>
       </c>
-      <c r="D5" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$3="",0,タスク一覧!$K$3-設定!$B$2)</f>
-        <v>0</v>
+      <c r="D5" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$3="",0,タスク一覧!$K$3)</f>
+        <v>46237</v>
       </c>
       <c r="E5" s="23" t="n">
         <f aca="false">IF(タスク一覧!$A$3="",0,IF(タスク一覧!$P$3="クリティカル",0,タスク一覧!$L$3-タスク一覧!$K$3+1))</f>
@@ -10821,9 +10855,9 @@
         <f aca="false">IF(タスク一覧!$A$4="","",タスク一覧!$L$4)</f>
         <v>46245</v>
       </c>
-      <c r="D6" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$4="",0,タスク一覧!$K$4-設定!$B$2)</f>
-        <v>3</v>
+      <c r="D6" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$4="",0,タスク一覧!$K$4)</f>
+        <v>46240</v>
       </c>
       <c r="E6" s="23" t="n">
         <f aca="false">IF(タスク一覧!$A$4="",0,IF(タスク一覧!$P$4="クリティカル",0,タスク一覧!$L$4-タスク一覧!$K$4+1))</f>
@@ -10847,9 +10881,9 @@
         <f aca="false">IF(タスク一覧!$A$5="","",タスク一覧!$L$5)</f>
         <v>46247</v>
       </c>
-      <c r="D7" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$5="",0,タスク一覧!$K$5-設定!$B$2)</f>
-        <v>9</v>
+      <c r="D7" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$5="",0,タスク一覧!$K$5)</f>
+        <v>46246</v>
       </c>
       <c r="E7" s="23" t="n">
         <f aca="false">IF(タスク一覧!$A$5="",0,IF(タスク一覧!$P$5="クリティカル",0,タスク一覧!$L$5-タスク一覧!$K$5+1))</f>
@@ -10873,9 +10907,9 @@
         <f aca="false">IF(タスク一覧!$A$6="","",タスク一覧!$L$6)</f>
         <v>46254</v>
       </c>
-      <c r="D8" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$6="",0,タスク一覧!$K$6-設定!$B$2)</f>
-        <v>11</v>
+      <c r="D8" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$6="",0,タスク一覧!$K$6)</f>
+        <v>46248</v>
       </c>
       <c r="E8" s="23" t="n">
         <f aca="false">IF(タスク一覧!$A$6="",0,IF(タスク一覧!$P$6="クリティカル",0,タスク一覧!$L$6-タスク一覧!$K$6+1))</f>
@@ -10899,9 +10933,9 @@
         <f aca="false">IF(タスク一覧!$A$7="","",タスク一覧!$L$7)</f>
         <v>46254</v>
       </c>
-      <c r="D9" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$7="",0,タスク一覧!$K$7-設定!$B$2)</f>
-        <v>11</v>
+      <c r="D9" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$7="",0,タスク一覧!$K$7)</f>
+        <v>46248</v>
       </c>
       <c r="E9" s="23" t="n">
         <f aca="false">IF(タスク一覧!$A$7="",0,IF(タスク一覧!$P$7="クリティカル",0,タスク一覧!$L$7-タスク一覧!$K$7+1))</f>
@@ -10925,9 +10959,9 @@
         <f aca="false">IF(タスク一覧!$A$8="","",タスク一覧!$L$8)</f>
         <v>46259</v>
       </c>
-      <c r="D10" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$8="",0,タスク一覧!$K$8-設定!$B$2)</f>
-        <v>18</v>
+      <c r="D10" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$8="",0,タスク一覧!$K$8)</f>
+        <v>46255</v>
       </c>
       <c r="E10" s="23" t="n">
         <f aca="false">IF(タスク一覧!$A$8="",0,IF(タスク一覧!$P$8="クリティカル",0,タスク一覧!$L$8-タスク一覧!$K$8+1))</f>
@@ -10951,9 +10985,9 @@
         <f aca="false">IF(タスク一覧!$A$9="","",タスク一覧!$L$9)</f>
         <v>46261</v>
       </c>
-      <c r="D11" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$9="",0,タスク一覧!$K$9-設定!$B$2)</f>
-        <v>23</v>
+      <c r="D11" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$9="",0,タスク一覧!$K$9)</f>
+        <v>46260</v>
       </c>
       <c r="E11" s="23" t="n">
         <f aca="false">IF(タスク一覧!$A$9="",0,IF(タスク一覧!$P$9="クリティカル",0,タスク一覧!$L$9-タスク一覧!$K$9+1))</f>
@@ -10977,9 +11011,9 @@
         <f aca="false">IF(タスク一覧!$A$10="","",タスク一覧!$L$10)</f>
         <v>46273</v>
       </c>
-      <c r="D12" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$10="",0,タスク一覧!$K$10-設定!$B$2)</f>
-        <v>25</v>
+      <c r="D12" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$10="",0,タスク一覧!$K$10)</f>
+        <v>46262</v>
       </c>
       <c r="E12" s="23" t="n">
         <f aca="false">IF(タスク一覧!$A$10="",0,IF(タスク一覧!$P$10="クリティカル",0,タスク一覧!$L$10-タスク一覧!$K$10+1))</f>
@@ -11003,9 +11037,9 @@
         <f aca="false">IF(タスク一覧!$A$11="","",タスク一覧!$L$11)</f>
         <v>46240</v>
       </c>
-      <c r="D13" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$11="",0,タスク一覧!$K$11-設定!$B$2)</f>
-        <v>0</v>
+      <c r="D13" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$11="",0,タスク一覧!$K$11)</f>
+        <v>46237</v>
       </c>
       <c r="E13" s="23" t="n">
         <f aca="false">IF(タスク一覧!$A$11="",0,IF(タスク一覧!$P$11="クリティカル",0,タスク一覧!$L$11-タスク一覧!$K$11+1))</f>
@@ -11029,9 +11063,9 @@
         <f aca="false">IF(タスク一覧!$A$12="","",タスク一覧!$L$12)</f>
         <v>46279</v>
       </c>
-      <c r="D14" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$12="",0,タスク一覧!$K$12-設定!$B$2)</f>
-        <v>37</v>
+      <c r="D14" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$12="",0,タスク一覧!$K$12)</f>
+        <v>46274</v>
       </c>
       <c r="E14" s="23" t="n">
         <f aca="false">IF(タスク一覧!$A$12="",0,IF(タスク一覧!$P$12="クリティカル",0,タスク一覧!$L$12-タスク一覧!$K$12+1))</f>
@@ -11055,9 +11089,9 @@
         <f aca="false">IF(タスク一覧!$A$13="","",タスク一覧!$L$13)</f>
         <v>46280</v>
       </c>
-      <c r="D15" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$13="",0,タスク一覧!$K$13-設定!$B$2)</f>
-        <v>43</v>
+      <c r="D15" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$13="",0,タスク一覧!$K$13)</f>
+        <v>46280</v>
       </c>
       <c r="E15" s="23" t="n">
         <f aca="false">IF(タスク一覧!$A$13="",0,IF(タスク一覧!$P$13="クリティカル",0,タスク一覧!$L$13-タスク一覧!$K$13+1))</f>
@@ -11081,8 +11115,8 @@
         <f aca="false">IF(タスク一覧!$A$14="","",タスク一覧!$L$14)</f>
         <v/>
       </c>
-      <c r="D16" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$14="",0,タスク一覧!$K$14-設定!$B$2)</f>
+      <c r="D16" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$14="",0,タスク一覧!$K$14)</f>
         <v>0</v>
       </c>
       <c r="E16" s="23" t="n">
@@ -11107,8 +11141,8 @@
         <f aca="false">IF(タスク一覧!$A$15="","",タスク一覧!$L$15)</f>
         <v/>
       </c>
-      <c r="D17" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$15="",0,タスク一覧!$K$15-設定!$B$2)</f>
+      <c r="D17" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$15="",0,タスク一覧!$K$15)</f>
         <v>0</v>
       </c>
       <c r="E17" s="23" t="n">
@@ -11133,8 +11167,8 @@
         <f aca="false">IF(タスク一覧!$A$16="","",タスク一覧!$L$16)</f>
         <v/>
       </c>
-      <c r="D18" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$16="",0,タスク一覧!$K$16-設定!$B$2)</f>
+      <c r="D18" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$16="",0,タスク一覧!$K$16)</f>
         <v>0</v>
       </c>
       <c r="E18" s="23" t="n">
@@ -11159,8 +11193,8 @@
         <f aca="false">IF(タスク一覧!$A$17="","",タスク一覧!$L$17)</f>
         <v/>
       </c>
-      <c r="D19" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$17="",0,タスク一覧!$K$17-設定!$B$2)</f>
+      <c r="D19" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$17="",0,タスク一覧!$K$17)</f>
         <v>0</v>
       </c>
       <c r="E19" s="23" t="n">
@@ -11185,8 +11219,8 @@
         <f aca="false">IF(タスク一覧!$A$18="","",タスク一覧!$L$18)</f>
         <v/>
       </c>
-      <c r="D20" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$18="",0,タスク一覧!$K$18-設定!$B$2)</f>
+      <c r="D20" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$18="",0,タスク一覧!$K$18)</f>
         <v>0</v>
       </c>
       <c r="E20" s="23" t="n">
@@ -11211,8 +11245,8 @@
         <f aca="false">IF(タスク一覧!$A$19="","",タスク一覧!$L$19)</f>
         <v/>
       </c>
-      <c r="D21" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$19="",0,タスク一覧!$K$19-設定!$B$2)</f>
+      <c r="D21" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$19="",0,タスク一覧!$K$19)</f>
         <v>0</v>
       </c>
       <c r="E21" s="23" t="n">
@@ -11237,8 +11271,8 @@
         <f aca="false">IF(タスク一覧!$A$20="","",タスク一覧!$L$20)</f>
         <v/>
       </c>
-      <c r="D22" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$20="",0,タスク一覧!$K$20-設定!$B$2)</f>
+      <c r="D22" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$20="",0,タスク一覧!$K$20)</f>
         <v>0</v>
       </c>
       <c r="E22" s="23" t="n">
@@ -11263,8 +11297,8 @@
         <f aca="false">IF(タスク一覧!$A$21="","",タスク一覧!$L$21)</f>
         <v/>
       </c>
-      <c r="D23" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$21="",0,タスク一覧!$K$21-設定!$B$2)</f>
+      <c r="D23" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$21="",0,タスク一覧!$K$21)</f>
         <v>0</v>
       </c>
       <c r="E23" s="23" t="n">
@@ -11289,8 +11323,8 @@
         <f aca="false">IF(タスク一覧!$A$22="","",タスク一覧!$L$22)</f>
         <v/>
       </c>
-      <c r="D24" s="23" t="n">
-        <f aca="false">IF(タスク一覧!$A$22="",0,タスク一覧!$K$22-設定!$B$2)</f>
+      <c r="D24" s="9" t="n">
+        <f aca="false">IF(タスク一覧!$A$22="",0,タスク一覧!$K$22)</f>
         <v>0</v>
       </c>
       <c r="E24" s="23" t="n">

</xml_diff>